<commit_message>
todays download csv files are 165+ and adding all to git and total graph data of csv are downloaded and we will start will table data now
</commit_message>
<xml_diff>
--- a/NZ_Sports_Data_Tracker.xlsx
+++ b/NZ_Sports_Data_Tracker.xlsx
@@ -1721,7 +1721,9 @@
       <c r="J11" s="22"/>
       <c r="K11" s="23"/>
       <c r="L11" s="23"/>
-      <c r="M11" s="24"/>
+      <c r="M11" s="24">
+        <v>502</v>
+      </c>
       <c r="N11" s="20" t="s">
         <v>42</v>
       </c>

</xml_diff>

<commit_message>
starting with 'Ministry of Health' data
</commit_message>
<xml_diff>
--- a/NZ_Sports_Data_Tracker.xlsx
+++ b/NZ_Sports_Data_Tracker.xlsx
@@ -809,6 +809,201 @@
   </cellStyleXfs>
   <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="18" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="19" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="20" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="22" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="24" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="26" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="28" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -817,201 +1012,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="16" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="17" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="18" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="19" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="20" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="24" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="26" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="28" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1323,7 +1323,7 @@
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="14" style="67" customWidth="1"/>
+    <col min="5" max="5" width="14" style="61" customWidth="1"/>
     <col min="6" max="6" width="80.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
@@ -1335,828 +1335,838 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="64"/>
     </row>
     <row r="3" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="64" t="s">
+      <c r="E3" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="N3" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="8">
+      <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="65" t="s">
+      <c r="E4" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="15"/>
-      <c r="K4" s="16">
+      <c r="J4" s="9"/>
+      <c r="K4" s="10">
         <v>46175</v>
       </c>
-      <c r="L4" s="16"/>
-      <c r="M4" s="17" t="s">
+      <c r="L4" s="10"/>
+      <c r="M4" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="N4" s="11" t="s">
+      <c r="N4" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="18">
+      <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="66" t="s">
+      <c r="E5" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="21" t="s">
+      <c r="F5" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="I5" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="22"/>
-      <c r="K5" s="16">
+      <c r="J5" s="16"/>
+      <c r="K5" s="10">
         <v>46175</v>
       </c>
-      <c r="L5" s="23"/>
-      <c r="M5" s="24" t="s">
+      <c r="L5" s="17"/>
+      <c r="M5" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="N5" s="20" t="s">
+      <c r="N5" s="14" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
+      <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="65" t="s">
+      <c r="E6" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="I6" s="25" t="s">
+      <c r="I6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="J6" s="15"/>
-      <c r="K6" s="16">
+      <c r="J6" s="9"/>
+      <c r="K6" s="10">
         <v>46175</v>
       </c>
-      <c r="L6" s="16"/>
-      <c r="M6" s="17" t="s">
+      <c r="L6" s="10"/>
+      <c r="M6" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="N6" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18">
+      <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="66" t="s">
+      <c r="E7" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="21" t="s">
+      <c r="F7" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="H7" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="I7" s="25" t="s">
+      <c r="I7" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="J7" s="22"/>
-      <c r="K7" s="16">
+      <c r="J7" s="16"/>
+      <c r="K7" s="10">
         <v>46175</v>
       </c>
-      <c r="L7" s="23"/>
-      <c r="M7" s="68" t="s">
+      <c r="L7" s="17"/>
+      <c r="M7" s="62" t="s">
         <v>141</v>
       </c>
-      <c r="N7" s="20" t="s">
+      <c r="N7" s="14" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+      <c r="A8" s="2">
         <v>5</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="65" t="s">
+      <c r="E8" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="I8" s="25" t="s">
+      <c r="I8" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="15"/>
-      <c r="K8" s="16">
+      <c r="J8" s="9"/>
+      <c r="K8" s="10">
         <v>46175</v>
       </c>
-      <c r="L8" s="16"/>
-      <c r="M8" s="68" t="s">
+      <c r="L8" s="10"/>
+      <c r="M8" s="62" t="s">
         <v>141</v>
       </c>
-      <c r="N8" s="11" t="s">
+      <c r="N8" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18">
+      <c r="A9" s="12">
         <v>6</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="66" t="s">
+      <c r="E9" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="21" t="s">
+      <c r="F9" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="I9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="J9" s="22"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="24" t="s">
+      <c r="J9" s="16"/>
+      <c r="K9" s="10">
+        <v>46175</v>
+      </c>
+      <c r="L9" s="17"/>
+      <c r="M9" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="N9" s="20" t="s">
+      <c r="N9" s="14" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8">
+      <c r="A10" s="2">
         <v>7</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="65" t="s">
+      <c r="E10" s="59" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="I10" s="14" t="s">
+      <c r="I10" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="J10" s="15"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="17" t="s">
+      <c r="J10" s="9"/>
+      <c r="K10" s="10">
+        <v>46175</v>
+      </c>
+      <c r="L10" s="10"/>
+      <c r="M10" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="N10" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="18">
+      <c r="A11" s="12">
         <v>8</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="66" t="s">
+      <c r="E11" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="26" t="s">
+      <c r="G11" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="J11" s="22"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="24">
+      <c r="J11" s="16"/>
+      <c r="K11" s="10">
+        <v>46175</v>
+      </c>
+      <c r="L11" s="17"/>
+      <c r="M11" s="18">
         <v>502</v>
       </c>
-      <c r="N11" s="20" t="s">
+      <c r="N11" s="14" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8">
+      <c r="A12" s="2">
         <v>9</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="65" t="s">
+      <c r="E12" s="59" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I12" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="J12" s="9"/>
+      <c r="K12" s="10">
+        <v>46175</v>
+      </c>
+      <c r="L12" s="10">
+        <v>46176</v>
+      </c>
+      <c r="M12" s="11"/>
+      <c r="N12" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12">
+        <v>10</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="60" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="I12" s="25" t="s">
+      <c r="I13" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="J12" s="15"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="18">
-        <v>10</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="E13" s="66" t="s">
+      <c r="J13" s="16"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
+      <c r="M13" s="18"/>
+      <c r="N13" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="59" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J14" s="9"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="12">
+        <v>12</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="60" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="J15" s="16"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="18"/>
+      <c r="N15" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="59" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I16" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="J16" s="9"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="12">
+        <v>14</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" s="60" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="J17" s="16"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="18"/>
+      <c r="N17" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="59" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J18" s="9"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="11"/>
+      <c r="N18" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12">
+        <v>16</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="60" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J19" s="16"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="17"/>
+      <c r="M19" s="18"/>
+      <c r="N19" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E20" s="59" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="J20" s="9"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="11"/>
+      <c r="N20" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="12">
+        <v>18</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="60" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="J21" s="16"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="18"/>
+      <c r="N21" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
         <v>19</v>
       </c>
-      <c r="F13" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="G13" s="10" t="s">
+      <c r="B22" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22" s="59" t="s">
+        <v>62</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H13" s="13" t="s">
+      <c r="H22" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="I13" s="25" t="s">
+      <c r="I22" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="J22" s="9"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="11"/>
+      <c r="N22" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="12">
+        <v>20</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="60" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I23" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="J13" s="22"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="24"/>
-      <c r="N13" s="20" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8">
-        <v>11</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="E14" s="65" t="s">
-        <v>40</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="G14" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="H14" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="J14" s="15"/>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="18">
-        <v>12</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" s="66" t="s">
-        <v>62</v>
-      </c>
-      <c r="F15" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I15" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="J15" s="22"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="24"/>
-      <c r="N15" s="20" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="8">
-        <v>13</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C16" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E16" s="65" t="s">
-        <v>62</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H16" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I16" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="J16" s="15"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="11" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="18">
-        <v>14</v>
-      </c>
-      <c r="B17" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="C17" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="E17" s="66" t="s">
-        <v>70</v>
-      </c>
-      <c r="F17" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I17" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="J17" s="22"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="24"/>
-      <c r="N17" s="20" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8">
-        <v>15</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18" s="65" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H18" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I18" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="J18" s="15"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="11" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="18">
-        <v>16</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="D19" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="E19" s="66" t="s">
-        <v>40</v>
-      </c>
-      <c r="F19" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="G19" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I19" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="J19" s="22"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="24"/>
-      <c r="N19" s="20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8">
-        <v>17</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="E20" s="65" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="G20" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I20" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="J20" s="15"/>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="18">
-        <v>18</v>
-      </c>
-      <c r="B21" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="D21" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="E21" s="66" t="s">
-        <v>40</v>
-      </c>
-      <c r="F21" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H21" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I21" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="J21" s="22"/>
-      <c r="K21" s="23"/>
-      <c r="L21" s="23"/>
-      <c r="M21" s="24"/>
-      <c r="N21" s="20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="8">
-        <v>19</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="C22" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" s="65" t="s">
-        <v>62</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H22" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I22" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="J22" s="15"/>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="11" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="18">
-        <v>20</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="E23" s="66" t="s">
-        <v>40</v>
-      </c>
-      <c r="F23" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="G23" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="H23" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I23" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="J23" s="22"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="24"/>
-      <c r="N23" s="20" t="s">
+      <c r="J23" s="16"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="18"/>
+      <c r="N23" s="14" t="s">
         <v>42</v>
       </c>
     </row>
@@ -2207,277 +2217,277 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="64" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
     </row>
     <row r="4" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="1" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="B5" s="30">
+      <c r="B5" s="24">
         <f>COUNTA('NZ Sports Data Tracker'!B4:B23)</f>
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="26">
         <f>K9</f>
         <v>0</v>
       </c>
-      <c r="C6" s="33">
+      <c r="C6" s="27">
         <f>B6/B5</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="35">
+      <c r="B7" s="29">
         <f>COUNTIF('NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
         <v>1</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="30">
         <f>B7/B5</f>
         <v>0.05</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="31" t="s">
         <v>106</v>
       </c>
-      <c r="B8" s="38">
+      <c r="B8" s="32">
         <f>COUNTIF('NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
-        <v>11</v>
-      </c>
-      <c r="C8" s="39">
+        <v>10</v>
+      </c>
+      <c r="C8" s="33">
         <f>B8/B5</f>
-        <v>0.55000000000000004</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="34" t="s">
         <v>107</v>
       </c>
-      <c r="B9" s="41">
+      <c r="B9" s="35">
         <f>COUNTIF('NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
         <v>4</v>
       </c>
-      <c r="C9" s="42">
+      <c r="C9" s="36">
         <f>B9/B5</f>
         <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="65" t="s">
         <v>108</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="65"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="1" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="43" t="s">
+      <c r="A13" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="44">
+      <c r="B13" s="38">
         <f>COUNTIF('NZ Sports Data Tracker'!C4:C23,"Participation")</f>
         <v>5</v>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="26">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Participation",'NZ Sports Data Tracker'!H4:H23,"Completed")</f>
         <v>4</v>
       </c>
-      <c r="D13" s="35">
+      <c r="D13" s="29">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Participation",'NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="E13" s="38">
+      <c r="E13" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Participation",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
         <v>0</v>
       </c>
-      <c r="F13" s="41">
+      <c r="F13" s="35">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Participation",'NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
         <v>1</v>
       </c>
-      <c r="G13" s="45">
+      <c r="G13" s="39">
         <f>IF(B13=0,"-",C13/B13)</f>
         <v>0.8</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="47">
+      <c r="B14" s="41">
         <f>COUNTIF('NZ Sports Data Tracker'!C4:C23,"Govt Open Data")</f>
         <v>5</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="26">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Govt Open Data",'NZ Sports Data Tracker'!H4:H23,"Completed")</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="35">
+        <v>1</v>
+      </c>
+      <c r="D14" s="29">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Govt Open Data",'NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
         <v>1</v>
       </c>
-      <c r="E14" s="38">
+      <c r="E14" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Govt Open Data",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
-        <v>1</v>
-      </c>
-      <c r="F14" s="41">
+        <v>0</v>
+      </c>
+      <c r="F14" s="35">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Govt Open Data",'NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
         <v>3</v>
       </c>
-      <c r="G14" s="48">
+      <c r="G14" s="42">
         <f>IF(B14=0,"-",C14/B14)</f>
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="49" t="s">
+      <c r="A15" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="50">
+      <c r="B15" s="44">
         <f>COUNTIF('NZ Sports Data Tracker'!C4:C23,"Rugby")</f>
         <v>4</v>
       </c>
-      <c r="C15" s="32">
+      <c r="C15" s="26">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Rugby",'NZ Sports Data Tracker'!H4:H23,"Completed")</f>
         <v>0</v>
       </c>
-      <c r="D15" s="35">
+      <c r="D15" s="29">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Rugby",'NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="E15" s="38">
+      <c r="E15" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Rugby",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
         <v>4</v>
       </c>
-      <c r="F15" s="41">
+      <c r="F15" s="35">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Rugby",'NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="G15" s="51">
+      <c r="G15" s="45">
         <f>IF(B15=0,"-",C15/B15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52" t="s">
+      <c r="A16" s="46" t="s">
         <v>76</v>
       </c>
-      <c r="B16" s="53">
+      <c r="B16" s="47">
         <f>COUNTIF('NZ Sports Data Tracker'!C4:C23,"Cricket")</f>
         <v>3</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="26">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Cricket",'NZ Sports Data Tracker'!H4:H23,"Completed")</f>
         <v>0</v>
       </c>
-      <c r="D16" s="35">
+      <c r="D16" s="29">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Cricket",'NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="E16" s="38">
+      <c r="E16" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Cricket",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
         <v>3</v>
       </c>
-      <c r="F16" s="41">
+      <c r="F16" s="35">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Cricket",'NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="G16" s="54">
+      <c r="G16" s="48">
         <f>IF(B16=0,"-",C16/B16)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="55" t="s">
+      <c r="A17" s="49" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="56">
+      <c r="B17" s="50">
         <f>COUNTIF('NZ Sports Data Tracker'!C4:C23,"Football")</f>
         <v>3</v>
       </c>
-      <c r="C17" s="32">
+      <c r="C17" s="26">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Football",'NZ Sports Data Tracker'!H4:H23,"Completed")</f>
         <v>0</v>
       </c>
-      <c r="D17" s="35">
+      <c r="D17" s="29">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Football",'NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="E17" s="38">
+      <c r="E17" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Football",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
         <v>3</v>
       </c>
-      <c r="F17" s="41">
+      <c r="F17" s="35">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Football",'NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="G17" s="57">
+      <c r="G17" s="51">
         <f>IF(B17=0,"-",C17/B17)</f>
         <v>0</v>
       </c>
@@ -2506,247 +2516,262 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="63" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
     </row>
     <row r="3" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
     </row>
     <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="67" t="s">
         <v>116</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
     </row>
     <row r="5" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="67" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="67"/>
     </row>
     <row r="6" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="67" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="67"/>
     </row>
     <row r="7" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="67" t="s">
         <v>119</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="C7" s="67"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="67"/>
     </row>
     <row r="9" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="68" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
+      <c r="B9" s="68"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="68"/>
+      <c r="E9" s="68"/>
     </row>
     <row r="10" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="67" t="s">
         <v>121</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+      <c r="C10" s="67"/>
+      <c r="D10" s="67"/>
+      <c r="E10" s="67"/>
     </row>
     <row r="11" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="59" t="s">
+      <c r="A11" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="67" t="s">
         <v>122</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="C11" s="67"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="67"/>
     </row>
     <row r="12" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="60" t="s">
+      <c r="A12" s="54" t="s">
         <v>73</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="67" t="s">
         <v>123</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="C12" s="67"/>
+      <c r="D12" s="67"/>
+      <c r="E12" s="67"/>
     </row>
     <row r="14" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="68" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
+      <c r="B14" s="68"/>
+      <c r="C14" s="68"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="68"/>
     </row>
     <row r="15" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="61" t="s">
+      <c r="A15" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="67" t="s">
         <v>125</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="C15" s="67"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="67"/>
     </row>
     <row r="16" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="62" t="s">
+      <c r="A16" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="67" t="s">
         <v>126</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="C16" s="67"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="67"/>
     </row>
     <row r="17" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="67" t="s">
         <v>127</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+      <c r="C17" s="67"/>
+      <c r="D17" s="67"/>
+      <c r="E17" s="67"/>
     </row>
     <row r="18" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="59" t="s">
+      <c r="A18" s="53" t="s">
         <v>76</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="67" t="s">
         <v>128</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="C18" s="67"/>
+      <c r="D18" s="67"/>
+      <c r="E18" s="67"/>
     </row>
     <row r="19" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="60" t="s">
+      <c r="A19" s="54" t="s">
         <v>89</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="67" t="s">
         <v>129</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
+      <c r="C19" s="67"/>
+      <c r="D19" s="67"/>
+      <c r="E19" s="67"/>
     </row>
     <row r="21" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="68" t="s">
         <v>130</v>
       </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
+      <c r="B21" s="68"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="68"/>
     </row>
     <row r="22" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="66" t="s">
         <v>131</v>
       </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
+      <c r="B22" s="66"/>
+      <c r="C22" s="66"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
     </row>
     <row r="23" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="66" t="s">
         <v>132</v>
       </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
+      <c r="B23" s="66"/>
+      <c r="C23" s="66"/>
+      <c r="D23" s="66"/>
+      <c r="E23" s="66"/>
     </row>
     <row r="24" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="66" t="s">
         <v>133</v>
       </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
     </row>
     <row r="25" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="66" t="s">
         <v>134</v>
       </c>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
+      <c r="B25" s="66"/>
+      <c r="C25" s="66"/>
+      <c r="D25" s="66"/>
+      <c r="E25" s="66"/>
     </row>
     <row r="26" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
     </row>
     <row r="27" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="66" t="s">
         <v>136</v>
       </c>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
+      <c r="B27" s="66"/>
+      <c r="C27" s="66"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
     </row>
     <row r="28" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="66" t="s">
         <v>137</v>
       </c>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
+      <c r="B28" s="66"/>
+      <c r="C28" s="66"/>
+      <c r="D28" s="66"/>
+      <c r="E28" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B18:E18"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A27:E27"/>
@@ -2756,21 +2781,6 @@
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
adding school NZ data and inside School data folder there are multiple folder which have multiple different source of data which is been stored as excel,csv,pdf and the remaining will be done by tomorrow inshallah
</commit_message>
<xml_diff>
--- a/NZ_Sports_Data_Tracker.xlsx
+++ b/NZ_Sports_Data_Tracker.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="152">
   <si>
     <t>🇳🇿  New Zealand Sports Data Sources — Integration Tracker</t>
   </si>
@@ -455,6 +455,33 @@
   </si>
   <si>
     <t>502 bad gateway</t>
+  </si>
+  <si>
+    <t>downloaded hug amount of data</t>
+  </si>
+  <si>
+    <t>downloaded excel and csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site not found </t>
+  </si>
+  <si>
+    <t>Just have html page and it shows normal data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">this site can't be reached </t>
+  </si>
+  <si>
+    <t>Not able to find any kind of excel related to NZ or any other country</t>
+  </si>
+  <si>
+    <t>Not able to find any kind of excel related to NZ or any other country or any free api from which we can go with</t>
+  </si>
+  <si>
+    <t>nothing just a static web page</t>
+  </si>
+  <si>
+    <t>The resource you are looking for is restricted and apparently not within your permissions. Please check your subscription.</t>
   </si>
 </sst>
 </file>
@@ -1004,13 +1031,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1330,7 +1357,7 @@
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
     <col min="11" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="35" customWidth="1"/>
+    <col min="13" max="13" width="35" style="61" customWidth="1"/>
     <col min="14" max="14" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1407,7 +1434,7 @@
       <c r="L3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" s="58" t="s">
         <v>14</v>
       </c>
       <c r="N3" s="1" t="s">
@@ -1769,7 +1796,9 @@
       <c r="L12" s="10">
         <v>46176</v>
       </c>
-      <c r="M12" s="11"/>
+      <c r="M12" s="11" t="s">
+        <v>143</v>
+      </c>
       <c r="N12" s="5" t="s">
         <v>52</v>
       </c>
@@ -1797,15 +1826,21 @@
         <v>21</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I13" s="19" t="s">
         <v>31</v>
       </c>
       <c r="J13" s="16"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
-      <c r="M13" s="18"/>
+      <c r="K13" s="10">
+        <v>46176</v>
+      </c>
+      <c r="L13" s="17">
+        <v>46177</v>
+      </c>
+      <c r="M13" s="18" t="s">
+        <v>144</v>
+      </c>
       <c r="N13" s="14" t="s">
         <v>24</v>
       </c>
@@ -1833,20 +1868,26 @@
         <v>59</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J14" s="9"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="11"/>
+      <c r="K14" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L14" s="17">
+        <v>46177</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>145</v>
+      </c>
       <c r="N14" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A15" s="12">
         <v>12</v>
       </c>
@@ -1869,15 +1910,21 @@
         <v>21</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>22</v>
+        <v>110</v>
       </c>
       <c r="I15" s="19" t="s">
         <v>31</v>
       </c>
       <c r="J15" s="16"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="17"/>
-      <c r="M15" s="18"/>
+      <c r="K15" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L15" s="17">
+        <v>46177</v>
+      </c>
+      <c r="M15" s="18" t="s">
+        <v>146</v>
+      </c>
       <c r="N15" s="14" t="s">
         <v>64</v>
       </c>
@@ -1905,15 +1952,21 @@
         <v>21</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I16" s="19" t="s">
         <v>31</v>
       </c>
       <c r="J16" s="9"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="11"/>
+      <c r="K16" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L16" s="17">
+        <v>46177</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>147</v>
+      </c>
       <c r="N16" s="5" t="s">
         <v>64</v>
       </c>
@@ -1941,20 +1994,24 @@
         <v>72</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I17" s="22" t="s">
         <v>73</v>
       </c>
       <c r="J17" s="16"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
+      <c r="K17" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L17" s="17">
+        <v>46177</v>
+      </c>
       <c r="M17" s="18"/>
       <c r="N17" s="14" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>15</v>
       </c>
@@ -1977,15 +2034,21 @@
         <v>21</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J18" s="9"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="11"/>
+      <c r="K18" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L18" s="17">
+        <v>46177</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>148</v>
+      </c>
       <c r="N18" s="5" t="s">
         <v>80</v>
       </c>
@@ -2013,15 +2076,21 @@
         <v>83</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J19" s="16"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="18"/>
+      <c r="K19" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L19" s="17">
+        <v>46177</v>
+      </c>
+      <c r="M19" s="18" t="s">
+        <v>149</v>
+      </c>
       <c r="N19" s="14" t="s">
         <v>42</v>
       </c>
@@ -2049,15 +2118,21 @@
         <v>21</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I20" s="19" t="s">
         <v>31</v>
       </c>
       <c r="J20" s="9"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="11"/>
+      <c r="K20" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L20" s="17">
+        <v>46177</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>150</v>
+      </c>
       <c r="N20" s="5" t="s">
         <v>87</v>
       </c>
@@ -2085,15 +2160,21 @@
         <v>21</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I21" s="19" t="s">
         <v>31</v>
       </c>
       <c r="J21" s="16"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="18"/>
+      <c r="K21" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L21" s="17">
+        <v>46177</v>
+      </c>
+      <c r="M21" s="62" t="s">
+        <v>151</v>
+      </c>
       <c r="N21" s="14" t="s">
         <v>42</v>
       </c>
@@ -2121,14 +2202,18 @@
         <v>21</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I22" s="22" t="s">
         <v>73</v>
       </c>
       <c r="J22" s="9"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
+      <c r="K22" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L22" s="17">
+        <v>46177</v>
+      </c>
       <c r="M22" s="11"/>
       <c r="N22" s="5" t="s">
         <v>64</v>
@@ -2157,14 +2242,18 @@
         <v>59</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="I23" s="19" t="s">
         <v>31</v>
       </c>
       <c r="J23" s="16"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
+      <c r="K23" s="17">
+        <v>46177</v>
+      </c>
+      <c r="L23" s="17">
+        <v>46177</v>
+      </c>
       <c r="M23" s="18"/>
       <c r="N23" s="14" t="s">
         <v>42</v>
@@ -2279,11 +2368,11 @@
       </c>
       <c r="B7" s="29">
         <f>COUNTIF('NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" s="30">
         <f>B7/B5</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2292,11 +2381,11 @@
       </c>
       <c r="B8" s="32">
         <f>COUNTIF('NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C8" s="33">
         <f>B8/B5</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2305,11 +2394,11 @@
       </c>
       <c r="B9" s="35">
         <f>COUNTIF('NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C9" s="36">
         <f>B9/B5</f>
-        <v>0.2</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2386,11 +2475,11 @@
       </c>
       <c r="C14" s="26">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Govt Open Data",'NZ Sports Data Tracker'!H4:H23,"Completed")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="29">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Govt Open Data",'NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Govt Open Data",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
@@ -2402,7 +2491,7 @@
       </c>
       <c r="G14" s="42">
         <f>IF(B14=0,"-",C14/B14)</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2415,7 +2504,7 @@
       </c>
       <c r="C15" s="26">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Rugby",'NZ Sports Data Tracker'!H4:H23,"Completed")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="29">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Rugby",'NZ Sports Data Tracker'!H4:H23,"In Progress")</f>
@@ -2423,15 +2512,15 @@
       </c>
       <c r="E15" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Rugby",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F15" s="35">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Rugby",'NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G15" s="45">
         <f>IF(B15=0,"-",C15/B15)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2452,11 +2541,11 @@
       </c>
       <c r="E16" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Cricket",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F16" s="35">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Cricket",'NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G16" s="48">
         <f>IF(B16=0,"-",C16/B16)</f>
@@ -2481,11 +2570,11 @@
       </c>
       <c r="E17" s="32">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Football",'NZ Sports Data Tracker'!H4:H23,"Not Started")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F17" s="35">
         <f>COUNTIFS('NZ Sports Data Tracker'!C4:C23,"Football",'NZ Sports Data Tracker'!H4:H23,"Blocked")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G17" s="51">
         <f>IF(B17=0,"-",C17/B17)</f>
@@ -2525,13 +2614,13 @@
       <c r="E1" s="63"/>
     </row>
     <row r="3" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="66" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
+      <c r="B3" s="66"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
     </row>
     <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="32" t="s">
@@ -2578,13 +2667,13 @@
       <c r="E7" s="67"/>
     </row>
     <row r="9" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="68" t="s">
+      <c r="A9" s="66" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="68"/>
-      <c r="C9" s="68"/>
-      <c r="D9" s="68"/>
-      <c r="E9" s="68"/>
+      <c r="B9" s="66"/>
+      <c r="C9" s="66"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
     </row>
     <row r="10" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="52" t="s">
@@ -2620,13 +2709,13 @@
       <c r="E12" s="67"/>
     </row>
     <row r="14" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="68" t="s">
+      <c r="A14" s="66" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="68"/>
-      <c r="C14" s="68"/>
-      <c r="D14" s="68"/>
-      <c r="E14" s="68"/>
+      <c r="B14" s="66"/>
+      <c r="C14" s="66"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="66"/>
     </row>
     <row r="15" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="55" t="s">
@@ -2684,94 +2773,79 @@
       <c r="E19" s="67"/>
     </row>
     <row r="21" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="68" t="s">
+      <c r="A21" s="66" t="s">
         <v>130</v>
       </c>
-      <c r="B21" s="68"/>
-      <c r="C21" s="68"/>
-      <c r="D21" s="68"/>
-      <c r="E21" s="68"/>
+      <c r="B21" s="66"/>
+      <c r="C21" s="66"/>
+      <c r="D21" s="66"/>
+      <c r="E21" s="66"/>
     </row>
     <row r="22" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="66" t="s">
+      <c r="A22" s="68" t="s">
         <v>131</v>
       </c>
-      <c r="B22" s="66"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
+      <c r="B22" s="68"/>
+      <c r="C22" s="68"/>
+      <c r="D22" s="68"/>
+      <c r="E22" s="68"/>
     </row>
     <row r="23" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="66" t="s">
+      <c r="A23" s="68" t="s">
         <v>132</v>
       </c>
-      <c r="B23" s="66"/>
-      <c r="C23" s="66"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
+      <c r="B23" s="68"/>
+      <c r="C23" s="68"/>
+      <c r="D23" s="68"/>
+      <c r="E23" s="68"/>
     </row>
     <row r="24" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="66" t="s">
+      <c r="A24" s="68" t="s">
         <v>133</v>
       </c>
-      <c r="B24" s="66"/>
-      <c r="C24" s="66"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="66"/>
+      <c r="B24" s="68"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
     </row>
     <row r="25" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="66" t="s">
+      <c r="A25" s="68" t="s">
         <v>134</v>
       </c>
-      <c r="B25" s="66"/>
-      <c r="C25" s="66"/>
-      <c r="D25" s="66"/>
-      <c r="E25" s="66"/>
+      <c r="B25" s="68"/>
+      <c r="C25" s="68"/>
+      <c r="D25" s="68"/>
+      <c r="E25" s="68"/>
     </row>
     <row r="26" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="66" t="s">
+      <c r="A26" s="68" t="s">
         <v>135</v>
       </c>
-      <c r="B26" s="66"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
+      <c r="B26" s="68"/>
+      <c r="C26" s="68"/>
+      <c r="D26" s="68"/>
+      <c r="E26" s="68"/>
     </row>
     <row r="27" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="68" t="s">
         <v>136</v>
       </c>
-      <c r="B27" s="66"/>
-      <c r="C27" s="66"/>
-      <c r="D27" s="66"/>
-      <c r="E27" s="66"/>
+      <c r="B27" s="68"/>
+      <c r="C27" s="68"/>
+      <c r="D27" s="68"/>
+      <c r="E27" s="68"/>
     </row>
     <row r="28" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="66" t="s">
+      <c r="A28" s="68" t="s">
         <v>137</v>
       </c>
-      <c r="B28" s="66"/>
-      <c r="C28" s="66"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="66"/>
+      <c r="B28" s="68"/>
+      <c r="C28" s="68"/>
+      <c r="D28" s="68"/>
+      <c r="E28" s="68"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A27:E27"/>
@@ -2781,6 +2855,21 @@
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Adding all downloaded file to github
</commit_message>
<xml_diff>
--- a/NZ_Sports_Data_Tracker.xlsx
+++ b/NZ_Sports_Data_Tracker.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="206">
   <si>
     <t>🇳🇿  New Zealand Sports Data Sources — Integration Tracker</t>
   </si>
@@ -482,6 +482,168 @@
   </si>
   <si>
     <t>The resource you are looking for is restricted and apparently not within your permissions. Please check your subscription.</t>
+  </si>
+  <si>
+    <t>Active NZ Survey 2024/25 (Latest Release)</t>
+  </si>
+  <si>
+    <t>https://sportnz.org.nz/resources/active-nz-survey-202425/</t>
+  </si>
+  <si>
+    <t>Voice of Rangatahi Survey 2023</t>
+  </si>
+  <si>
+    <t>Sport NZ / Youth</t>
+  </si>
+  <si>
+    <t>Voice of Participant Survey (Club Members)</t>
+  </si>
+  <si>
+    <t>Sport NZ / Clubs</t>
+  </si>
+  <si>
+    <t>School Sport NZ — Annual Census (2000–2024)</t>
+  </si>
+  <si>
+    <t>School Sport</t>
+  </si>
+  <si>
+    <t>Secondary School Sport</t>
+  </si>
+  <si>
+    <t>PDF + Excel Download</t>
+  </si>
+  <si>
+    <t>https://www.schoolsportnz.org.nz/Education/school-sport-nz-census-reports</t>
+  </si>
+  <si>
+    <t>MCH — Sport &amp; Recreation Industry Profile 2024 (Infometrics)</t>
+  </si>
+  <si>
+    <t>PDF Download</t>
+  </si>
+  <si>
+    <t>https://www.mch.govt.nz/sites/default/files/2025-03/sport-and-recreation-industry-profile-2024.pdf</t>
+  </si>
+  <si>
+    <t>Stats NZ — 2023 Census Data (Sport/Recreation filter)</t>
+  </si>
+  <si>
+    <t>https://www.stats.govt.nz/topics/census/</t>
+  </si>
+  <si>
+    <t>Stats NZ — Wellbeing Data (100 Indicators)</t>
+  </si>
+  <si>
+    <t>https://www.stats.govt.nz/indicators/wellbeing-statistics/</t>
+  </si>
+  <si>
+    <t>ACC — Sport Injury Claims Data (Sportwise)</t>
+  </si>
+  <si>
+    <t>Health/Research</t>
+  </si>
+  <si>
+    <t>Cross-sport NZ</t>
+  </si>
+  <si>
+    <t>https://www.acc.co.nz/sportwise</t>
+  </si>
+  <si>
+    <t>Sport &amp; Recreation Knowledge Library (srknowledge.org.nz)</t>
+  </si>
+  <si>
+    <t>Web Search / PDF</t>
+  </si>
+  <si>
+    <t>https://www.srknowledge.org.nz/</t>
+  </si>
+  <si>
+    <t>downloaded</t>
+  </si>
+  <si>
+    <t>Excel (.xlsx) + PDF</t>
+  </si>
+  <si>
+    <t>done</t>
+  </si>
+  <si>
+    <t>PDF (tables extractable)</t>
+  </si>
+  <si>
+    <t>nothing available</t>
+  </si>
+  <si>
+    <t>Excel / CSV</t>
+  </si>
+  <si>
+    <t>CSV / Excel</t>
+  </si>
+  <si>
+    <t>PDF / Reports</t>
+  </si>
+  <si>
+    <t>AUT Statistical Data Guide — Sport &amp; Recreation</t>
+  </si>
+  <si>
+    <t>Web (Discovery Hub)</t>
+  </si>
+  <si>
+    <t>https://aut.ac.nz.libguides.com/find_statistical_data/sport_and_rec</t>
+  </si>
+  <si>
+    <t>Downloaded pdf and excels  tried to read medallion architecture</t>
+  </si>
+  <si>
+    <t>Various (links hub)</t>
+  </si>
+  <si>
+    <t>NZ Cricket — Annual Reports &amp; Statistics</t>
+  </si>
+  <si>
+    <t>https://www.nzc.nz/about/annual-reports</t>
+  </si>
+  <si>
+    <t>PDF (tables)</t>
+  </si>
+  <si>
+    <t>NZ Rugby (NZR) — Official Stats &amp; Reports</t>
+  </si>
+  <si>
+    <t>All Blacks / NZ Rugby</t>
+  </si>
+  <si>
+    <t>Web Scrape / PDF</t>
+  </si>
+  <si>
+    <t>https://www.nzrugby.co.nz</t>
+  </si>
+  <si>
+    <t>PDF / HTML</t>
+  </si>
+  <si>
+    <t>Paralympics New Zealand — Disability Sport Data</t>
+  </si>
+  <si>
+    <t>Disability Sport NZ</t>
+  </si>
+  <si>
+    <t>https://www.paralympics.org.nz</t>
+  </si>
+  <si>
+    <t>Knowledge Auckland — Sport &amp; Recreation Reports</t>
+  </si>
+  <si>
+    <t>Auckland Region</t>
+  </si>
+  <si>
+    <t>https://www.knowledgeauckland.org.nz</t>
+  </si>
+  <si>
+    <t>PDF / Excel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO data found in that </t>
   </si>
 </sst>
 </file>
@@ -491,7 +653,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -707,8 +869,22 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -793,8 +969,20 @@
         <bgColor rgb="FFF7F6F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF0CC"/>
+        <bgColor rgb="FFFAEEDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4EC"/>
+        <bgColor rgb="FFFCE8E8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -830,11 +1018,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1031,20 +1235,195 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="15">
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF7C1D1D"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE8E8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF0C447C"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE6F1FB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF1A5C30"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD6F4E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF7C1D1D"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE8E8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF0C447C"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE6F1FB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF1A5C30"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD6F4E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF7C1D1D"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE8E8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF0C447C"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE6F1FB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF1A5C30"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD6F4E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF7C1D1D"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE8E8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF0C447C"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE6F1FB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF1A5C30"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD6F4E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <sz val="10"/>
@@ -1344,7 +1723,7 @@
   <sheetPr>
     <tabColor rgb="FF0D1B2A"/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1354,11 +1733,11 @@
     <col min="6" max="6" width="80.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="12" width="14" customWidth="1"/>
+    <col min="9" max="9" width="10" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="16" hidden="1" customWidth="1"/>
+    <col min="11" max="12" width="14" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="35" style="61" customWidth="1"/>
-    <col min="14" max="14" width="13" customWidth="1"/>
+    <col min="14" max="14" width="13" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2259,24 +2638,603 @@
         <v>42</v>
       </c>
     </row>
+    <row r="24" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="69">
+        <v>21</v>
+      </c>
+      <c r="B24" s="69" t="s">
+        <v>152</v>
+      </c>
+      <c r="C24" s="70" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="69" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="69" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="69" t="s">
+        <v>153</v>
+      </c>
+      <c r="G24" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I24" s="75" t="s">
+        <v>23</v>
+      </c>
+      <c r="J24" s="69"/>
+      <c r="K24" s="69"/>
+      <c r="L24" s="69"/>
+      <c r="M24" s="69" t="s">
+        <v>177</v>
+      </c>
+      <c r="N24" s="69" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A25" s="69">
+        <v>22</v>
+      </c>
+      <c r="B25" s="69" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" s="70" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="69" t="s">
+        <v>155</v>
+      </c>
+      <c r="E25" s="69" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="69" t="s">
+        <v>36</v>
+      </c>
+      <c r="G25" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I25" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="J25" s="69"/>
+      <c r="K25" s="69"/>
+      <c r="L25" s="69"/>
+      <c r="M25" s="76">
+        <v>404</v>
+      </c>
+      <c r="N25" s="69" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="69">
+        <v>23</v>
+      </c>
+      <c r="B26" s="69" t="s">
+        <v>156</v>
+      </c>
+      <c r="C26" s="70" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="69" t="s">
+        <v>157</v>
+      </c>
+      <c r="E26" s="69" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="71" t="s">
+        <v>34</v>
+      </c>
+      <c r="G26" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I26" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="J26" s="69"/>
+      <c r="K26" s="69"/>
+      <c r="L26" s="69"/>
+      <c r="M26" s="76">
+        <v>404</v>
+      </c>
+      <c r="N26" s="69" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="69">
+        <v>24</v>
+      </c>
+      <c r="B27" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="C27" s="72" t="s">
+        <v>159</v>
+      </c>
+      <c r="D27" s="69" t="s">
+        <v>160</v>
+      </c>
+      <c r="E27" s="69" t="s">
+        <v>161</v>
+      </c>
+      <c r="F27" s="69" t="s">
+        <v>162</v>
+      </c>
+      <c r="G27" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I27" s="75" t="s">
+        <v>23</v>
+      </c>
+      <c r="J27" s="69"/>
+      <c r="K27" s="69"/>
+      <c r="L27" s="69"/>
+      <c r="M27" s="69" t="s">
+        <v>179</v>
+      </c>
+      <c r="N27" s="69" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A28" s="69">
+        <v>25</v>
+      </c>
+      <c r="B28" s="69" t="s">
+        <v>163</v>
+      </c>
+      <c r="C28" s="73" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" s="69" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28" s="69" t="s">
+        <v>164</v>
+      </c>
+      <c r="F28" s="69" t="s">
+        <v>165</v>
+      </c>
+      <c r="G28" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I28" s="75" t="s">
+        <v>23</v>
+      </c>
+      <c r="J28" s="69"/>
+      <c r="K28" s="69"/>
+      <c r="L28" s="69"/>
+      <c r="M28" s="69" t="s">
+        <v>179</v>
+      </c>
+      <c r="N28" s="69" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A29" s="69">
+        <v>26</v>
+      </c>
+      <c r="B29" s="69" t="s">
+        <v>166</v>
+      </c>
+      <c r="C29" s="73" t="s">
+        <v>38</v>
+      </c>
+      <c r="D29" s="69" t="s">
+        <v>39</v>
+      </c>
+      <c r="E29" s="69" t="s">
+        <v>44</v>
+      </c>
+      <c r="F29" s="69" t="s">
+        <v>167</v>
+      </c>
+      <c r="G29" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I29" s="75" t="s">
+        <v>23</v>
+      </c>
+      <c r="J29" s="69"/>
+      <c r="K29" s="69"/>
+      <c r="L29" s="69"/>
+      <c r="M29" s="69" t="s">
+        <v>181</v>
+      </c>
+      <c r="N29" s="69" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A30" s="69">
+        <v>27</v>
+      </c>
+      <c r="B30" s="69" t="s">
+        <v>168</v>
+      </c>
+      <c r="C30" s="73" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="69" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="69" t="s">
+        <v>50</v>
+      </c>
+      <c r="F30" s="69" t="s">
+        <v>169</v>
+      </c>
+      <c r="G30" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I30" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="J30" s="69"/>
+      <c r="K30" s="69"/>
+      <c r="L30" s="69"/>
+      <c r="M30" s="69" t="s">
+        <v>181</v>
+      </c>
+      <c r="N30" s="69" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A31" s="69">
+        <v>28</v>
+      </c>
+      <c r="B31" s="69" t="s">
+        <v>170</v>
+      </c>
+      <c r="C31" s="74" t="s">
+        <v>171</v>
+      </c>
+      <c r="D31" s="69" t="s">
+        <v>172</v>
+      </c>
+      <c r="E31" s="69" t="s">
+        <v>50</v>
+      </c>
+      <c r="F31" s="69" t="s">
+        <v>173</v>
+      </c>
+      <c r="G31" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I31" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="J31" s="69"/>
+      <c r="K31" s="69"/>
+      <c r="L31" s="69"/>
+      <c r="M31" s="69" t="s">
+        <v>181</v>
+      </c>
+      <c r="N31" s="69" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="69">
+        <v>29</v>
+      </c>
+      <c r="B32" s="69" t="s">
+        <v>174</v>
+      </c>
+      <c r="C32" s="74" t="s">
+        <v>171</v>
+      </c>
+      <c r="D32" s="69" t="s">
+        <v>18</v>
+      </c>
+      <c r="E32" s="69" t="s">
+        <v>175</v>
+      </c>
+      <c r="F32" s="69" t="s">
+        <v>176</v>
+      </c>
+      <c r="G32" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I32" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="J32" s="69"/>
+      <c r="K32" s="69"/>
+      <c r="L32" s="69"/>
+      <c r="M32" s="69" t="s">
+        <v>181</v>
+      </c>
+      <c r="N32" s="69" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="69">
+        <v>30</v>
+      </c>
+      <c r="B33" s="69" t="s">
+        <v>185</v>
+      </c>
+      <c r="C33" s="74" t="s">
+        <v>171</v>
+      </c>
+      <c r="D33" s="69" t="s">
+        <v>172</v>
+      </c>
+      <c r="E33" s="69" t="s">
+        <v>186</v>
+      </c>
+      <c r="F33" s="69" t="s">
+        <v>187</v>
+      </c>
+      <c r="G33" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I33" s="69" t="s">
+        <v>73</v>
+      </c>
+      <c r="J33" s="69"/>
+      <c r="K33" s="69"/>
+      <c r="L33" s="69"/>
+      <c r="M33" s="69" t="s">
+        <v>188</v>
+      </c>
+      <c r="N33" s="69" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A34" s="69">
+        <v>31</v>
+      </c>
+      <c r="B34" s="69" t="s">
+        <v>190</v>
+      </c>
+      <c r="C34" s="77" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" s="69" t="s">
+        <v>85</v>
+      </c>
+      <c r="E34" s="69" t="s">
+        <v>164</v>
+      </c>
+      <c r="F34" s="69" t="s">
+        <v>191</v>
+      </c>
+      <c r="G34" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="I34" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="J34" s="69"/>
+      <c r="K34" s="69"/>
+      <c r="L34" s="69"/>
+      <c r="M34" s="76">
+        <v>404</v>
+      </c>
+      <c r="N34" s="69" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="69">
+        <v>32</v>
+      </c>
+      <c r="B35" s="69" t="s">
+        <v>193</v>
+      </c>
+      <c r="C35" s="78" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" s="69" t="s">
+        <v>194</v>
+      </c>
+      <c r="E35" s="69" t="s">
+        <v>195</v>
+      </c>
+      <c r="F35" s="69" t="s">
+        <v>196</v>
+      </c>
+      <c r="G35" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="I35" s="69" t="s">
+        <v>31</v>
+      </c>
+      <c r="J35" s="69"/>
+      <c r="K35" s="69"/>
+      <c r="L35" s="69"/>
+      <c r="M35" s="69" t="s">
+        <v>205</v>
+      </c>
+      <c r="N35" s="69" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A36" s="69">
+        <v>33</v>
+      </c>
+      <c r="B36" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="C36" s="70" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="69" t="s">
+        <v>199</v>
+      </c>
+      <c r="E36" s="69" t="s">
+        <v>164</v>
+      </c>
+      <c r="F36" s="69" t="s">
+        <v>200</v>
+      </c>
+      <c r="G36" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="I36" s="69" t="s">
+        <v>73</v>
+      </c>
+      <c r="J36" s="69"/>
+      <c r="K36" s="69"/>
+      <c r="L36" s="69"/>
+      <c r="M36" s="69" t="s">
+        <v>205</v>
+      </c>
+      <c r="N36" s="69" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A37" s="69">
+        <v>34</v>
+      </c>
+      <c r="B37" s="69" t="s">
+        <v>201</v>
+      </c>
+      <c r="C37" s="73" t="s">
+        <v>38</v>
+      </c>
+      <c r="D37" s="69" t="s">
+        <v>202</v>
+      </c>
+      <c r="E37" s="69" t="s">
+        <v>164</v>
+      </c>
+      <c r="F37" s="69" t="s">
+        <v>203</v>
+      </c>
+      <c r="G37" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="I37" s="69" t="s">
+        <v>73</v>
+      </c>
+      <c r="J37" s="69"/>
+      <c r="K37" s="69"/>
+      <c r="L37" s="69"/>
+      <c r="M37" s="69" t="s">
+        <v>205</v>
+      </c>
+      <c r="N37" s="69" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M38" s="69"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A4:N23">
-    <cfRule type="expression" dxfId="2" priority="2">
+  <conditionalFormatting sqref="A4:N23 H34:H36">
+    <cfRule type="expression" dxfId="14" priority="26">
       <formula>$H4="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="13" priority="27">
       <formula>$H4="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="12" priority="28">
       <formula>$H4="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H24:H31">
+    <cfRule type="expression" dxfId="11" priority="22">
+      <formula>$H24="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="23">
+      <formula>$H24="In Progress"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="24">
+      <formula>$H24="Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H32">
+    <cfRule type="expression" dxfId="8" priority="16">
+      <formula>$H32="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="17">
+      <formula>$H32="In Progress"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="18">
+      <formula>$H32="Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="expression" dxfId="5" priority="4">
+      <formula>$H37="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>$H37="In Progress"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="6">
+      <formula>$H37="Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H33">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>$H33="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$H33="In Progress"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>$H33="Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" errorTitle="Invalid status" error="Choose from: Not Started, In Progress, Completed, Blocked" sqref="H4:H23">
+    <dataValidation type="list" errorTitle="Invalid status" error="Choose from: Not Started, In Progress, Completed, Blocked" sqref="H4:H37">
       <formula1>"Not Started,In Progress,Completed,Blocked"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2285,8 +3243,11 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="F26" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2614,13 +3575,13 @@
       <c r="E1" s="63"/>
     </row>
     <row r="3" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="66" t="s">
+      <c r="A3" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
     </row>
     <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="32" t="s">
@@ -2667,13 +3628,13 @@
       <c r="E7" s="67"/>
     </row>
     <row r="9" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="66" t="s">
+      <c r="A9" s="68" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="66"/>
-      <c r="C9" s="66"/>
-      <c r="D9" s="66"/>
-      <c r="E9" s="66"/>
+      <c r="B9" s="68"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="68"/>
+      <c r="E9" s="68"/>
     </row>
     <row r="10" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="52" t="s">
@@ -2709,13 +3670,13 @@
       <c r="E12" s="67"/>
     </row>
     <row r="14" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="66" t="s">
+      <c r="A14" s="68" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="66"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
+      <c r="B14" s="68"/>
+      <c r="C14" s="68"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="68"/>
     </row>
     <row r="15" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="55" t="s">
@@ -2773,79 +3734,94 @@
       <c r="E19" s="67"/>
     </row>
     <row r="21" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="66" t="s">
+      <c r="A21" s="68" t="s">
         <v>130</v>
       </c>
-      <c r="B21" s="66"/>
-      <c r="C21" s="66"/>
-      <c r="D21" s="66"/>
-      <c r="E21" s="66"/>
+      <c r="B21" s="68"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="68"/>
     </row>
     <row r="22" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="68" t="s">
+      <c r="A22" s="66" t="s">
         <v>131</v>
       </c>
-      <c r="B22" s="68"/>
-      <c r="C22" s="68"/>
-      <c r="D22" s="68"/>
-      <c r="E22" s="68"/>
+      <c r="B22" s="66"/>
+      <c r="C22" s="66"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
     </row>
     <row r="23" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="68" t="s">
+      <c r="A23" s="66" t="s">
         <v>132</v>
       </c>
-      <c r="B23" s="68"/>
-      <c r="C23" s="68"/>
-      <c r="D23" s="68"/>
-      <c r="E23" s="68"/>
+      <c r="B23" s="66"/>
+      <c r="C23" s="66"/>
+      <c r="D23" s="66"/>
+      <c r="E23" s="66"/>
     </row>
     <row r="24" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="68" t="s">
+      <c r="A24" s="66" t="s">
         <v>133</v>
       </c>
-      <c r="B24" s="68"/>
-      <c r="C24" s="68"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="68"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
     </row>
     <row r="25" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="68" t="s">
+      <c r="A25" s="66" t="s">
         <v>134</v>
       </c>
-      <c r="B25" s="68"/>
-      <c r="C25" s="68"/>
-      <c r="D25" s="68"/>
-      <c r="E25" s="68"/>
+      <c r="B25" s="66"/>
+      <c r="C25" s="66"/>
+      <c r="D25" s="66"/>
+      <c r="E25" s="66"/>
     </row>
     <row r="26" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="68" t="s">
+      <c r="A26" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="B26" s="68"/>
-      <c r="C26" s="68"/>
-      <c r="D26" s="68"/>
-      <c r="E26" s="68"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
     </row>
     <row r="27" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="68" t="s">
+      <c r="A27" s="66" t="s">
         <v>136</v>
       </c>
-      <c r="B27" s="68"/>
-      <c r="C27" s="68"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="68"/>
+      <c r="B27" s="66"/>
+      <c r="C27" s="66"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
     </row>
     <row r="28" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="68" t="s">
+      <c r="A28" s="66" t="s">
         <v>137</v>
       </c>
-      <c r="B28" s="68"/>
-      <c r="C28" s="68"/>
-      <c r="D28" s="68"/>
-      <c r="E28" s="68"/>
+      <c r="B28" s="66"/>
+      <c r="C28" s="66"/>
+      <c r="D28" s="66"/>
+      <c r="E28" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B18:E18"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A27:E27"/>
@@ -2855,21 +3831,6 @@
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>